<commit_message>
security: scrub public repository artifacts
</commit_message>
<xml_diff>
--- a/client-report/client-directory-report.xlsx
+++ b/client-report/client-directory-report.xlsx
@@ -986,7 +986,7 @@
     <t>VERIFIED_SUCCESS: профиль создан и публично доступен (18+ млн бизнесов в каталоге)</t>
   </si>
   <si>
-    <t>VERIFIED_SUCCESS: Профиль создан и публично доступен. URL: https://www.find-us-here.com/businesses/Itllect-LLC-Plantation-Florida-USA/34578398/. Аккаунт: itllect / DimaItllect2026!55. Заполнены: контакты, адрес, категория (Advertising - Direct Mail), описание. Email verification не требуется (аккаунт активирован сразу).</t>
+    <t>VERIFIED_SUCCESS: Профиль создан и публично доступен. URL: https://www.find-us-here.com/businesses/Itllect-LLC-Plantation-Florida-USA/34578398/. Аккаунт: itllect / [REDACTED]. Заполнены: контакты, адрес, категория (Advertising - Direct Mail), описание. Email verification не требуется (аккаунт активирован сразу).</t>
   </si>
   <si>
     <t>Подтверждено в headed-сессии 31.07 (turnstile решён, submit прошёл)</t>
@@ -1028,7 +1028,7 @@
     <t>VERIFIED_SUCCESS: профиль создан и публично доступен</t>
   </si>
   <si>
-    <t>VERIFIED_SUCCESS: Профиль создан и подтверждён. URL: https://www.semfirms.com/profile/itllect-llc. Аккаунт: itllect.marketing@gmail.com / DimaItllect2026!55. Блокировало: поле title требовало 'Itllect LLC' (полное юридическое название). Drupal валидация отклоняла форму без полного названия компании.</t>
+    <t>VERIFIED_SUCCESS: Профиль создан и подтверждён. URL: https://www.semfirms.com/profile/itllect-llc. Аккаунт: itllect.marketing@gmail.com / [REDACTED]. Блокировало: поле title требовало 'Itllect LLC' (полное юридическое название). Drupal валидация отклоняла форму без полного названия компании.</t>
   </si>
   <si>
     <t>Форма жива на /registration (Drupal); заполнение проходит, submit зависает — нужен ручной шаг</t>
@@ -1786,7 +1786,7 @@
     <mergeCell ref="A28:C31"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -4241,7 +4241,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -4888,7 +4888,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -5269,7 +5269,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -7037,6 +7037,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>